<commit_message>
Add per-location pull priority to PullList
Locations gains a PullPriority column (1 = pull from here first).
Default order: Prep -> Sauté -> Walk-in -> Dry -> Freezer.

PullList now walks an item's locations in priority order and greedily
allocates the requisition's portion need across them via a self-SUMIFS
on PortionsToPullHere with PullPriority < current row. Output columns
make the cook's job explicit: PortionsToPullHere and StillShortAfterHere
per location.
</commit_message>
<xml_diff>
--- a/templates/restaurant-boh-inventory.xlsx
+++ b/templates/restaurant-boh-inventory.xlsx
@@ -174,12 +174,13 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="tbl_Locations" displayName="tbl_Locations" ref="A1:C6" headerRowCount="1">
-  <autoFilter ref="A1:C6"/>
-  <tableColumns count="3">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="tbl_Locations" displayName="tbl_Locations" ref="A1:D6" headerRowCount="1">
+  <autoFilter ref="A1:D6"/>
+  <tableColumns count="4">
     <tableColumn id="1" name="LocationCode"/>
     <tableColumn id="2" name="LocationName"/>
     <tableColumn id="3" name="Zone"/>
+    <tableColumn id="4" name="PullPriority"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -236,16 +237,20 @@
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="tbl_PullList" displayName="tbl_PullList" ref="A1:G17" headerRowCount="1">
-  <autoFilter ref="A1:G17"/>
-  <tableColumns count="7">
-    <tableColumn id="1" name="LocationCode"/>
-    <tableColumn id="2" name="LocationName"/>
-    <tableColumn id="3" name="ItemCode"/>
-    <tableColumn id="4" name="ItemName"/>
-    <tableColumn id="5" name="PortionsAvailable"/>
-    <tableColumn id="6" name="PortionUOM"/>
-    <tableColumn id="7" name="PortionsNeededForRequisition"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="tbl_PullList" displayName="tbl_PullList" ref="A1:K17" headerRowCount="1">
+  <autoFilter ref="A1:K17"/>
+  <tableColumns count="11">
+    <tableColumn id="1" name="ItemCode"/>
+    <tableColumn id="2" name="ItemName"/>
+    <tableColumn id="3" name="LocationCode"/>
+    <tableColumn id="4" name="LocationName"/>
+    <tableColumn id="5" name="PullPriority"/>
+    <tableColumn id="6" name="PortionsAvailable"/>
+    <tableColumn id="7" name="PortionUOM"/>
+    <tableColumn id="8" name="PortionsNeededTotal"/>
+    <tableColumn id="9" name="AlreadyAllocatedHigherPriority"/>
+    <tableColumn id="10" name="PortionsToPullHere"/>
+    <tableColumn id="11" name="StillShortAfterHere"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -573,7 +578,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Locations    - storage locations (Walk-in, Freezer, etc.).</t>
+          <t xml:space="preserve">  Locations    - storage locations + PullPriority (1 = pull from here first).</t>
         </is>
       </c>
     </row>
@@ -601,7 +606,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t xml:space="preserve">  PullList     - which locations have stock for the items you need.</t>
+          <t xml:space="preserve">  PullList     - allocates the requisition across locations in PullPriority order.</t>
         </is>
       </c>
     </row>
@@ -1197,12 +1202,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C6"/>
+  <dimension ref="A1:D6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1221,90 +1227,110 @@
           <t>Zone</t>
         </is>
       </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>PullPriority</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>WALKIN</t>
+          <t>PREP</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Walk-in Cooler</t>
+          <t>Prep Station</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Cold</t>
-        </is>
+          <t>Prep</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>FRZ</t>
+          <t>SAUTE</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Freezer</t>
+          <t>Sauté Line</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Cold</t>
-        </is>
+          <t>Hot Line</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>DRY</t>
+          <t>WALKIN</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Dry Storage</t>
+          <t>Walk-in Cooler</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Ambient</t>
-        </is>
+          <t>Cold</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>SAUTE</t>
+          <t>DRY</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Sauté Line</t>
+          <t>Dry Storage</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Hot Line</t>
-        </is>
+          <t>Ambient</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>4</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>PREP</t>
+          <t>FRZ</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Prep Station</t>
+          <t>Freezer</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Prep</t>
-        </is>
+          <t>Cold</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>5</v>
       </c>
     </row>
   </sheetData>
@@ -2785,548 +2811,828 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G17"/>
+  <dimension ref="A1:K17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="22" customWidth="1" min="4" max="4"/>
-    <col width="19" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="30" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="19" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="21" customWidth="1" min="8" max="8"/>
+    <col width="32" customWidth="1" min="9" max="9"/>
+    <col width="20" customWidth="1" min="10" max="10"/>
+    <col width="21" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
+          <t>ItemCode</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>ItemName</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
           <t>LocationCode</t>
         </is>
       </c>
-      <c r="B1" s="2" t="inlineStr">
+      <c r="D1" s="2" t="inlineStr">
         <is>
           <t>LocationName</t>
         </is>
       </c>
-      <c r="C1" s="2" t="inlineStr">
-        <is>
-          <t>ItemCode</t>
-        </is>
-      </c>
-      <c r="D1" s="2" t="inlineStr">
-        <is>
-          <t>ItemName</t>
-        </is>
-      </c>
       <c r="E1" s="2" t="inlineStr">
         <is>
+          <t>PullPriority</t>
+        </is>
+      </c>
+      <c r="F1" s="2" t="inlineStr">
+        <is>
           <t>PortionsAvailable</t>
         </is>
       </c>
-      <c r="F1" s="2" t="inlineStr">
+      <c r="G1" s="2" t="inlineStr">
         <is>
           <t>PortionUOM</t>
         </is>
       </c>
-      <c r="G1" s="2" t="inlineStr">
-        <is>
-          <t>PortionsNeededForRequisition</t>
+      <c r="H1" s="2" t="inlineStr">
+        <is>
+          <t>PortionsNeededTotal</t>
+        </is>
+      </c>
+      <c r="I1" s="2" t="inlineStr">
+        <is>
+          <t>AlreadyAllocatedHigherPriority</t>
+        </is>
+      </c>
+      <c r="J1" s="2" t="inlineStr">
+        <is>
+          <t>PortionsToPullHere</t>
+        </is>
+      </c>
+      <c r="K1" s="2" t="inlineStr">
+        <is>
+          <t>StillShortAfterHere</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>WALKIN</t>
+          <t>BUTTER</t>
         </is>
       </c>
       <c r="B2">
-        <f>XLOOKUP(A2, tbl_Locations[LocationCode], tbl_Locations[LocationName], "")</f>
+        <f>XLOOKUP(A2, tbl_Items[ItemCode], tbl_Items[ItemName], "")</f>
         <v/>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>PORK-CHOP-6OZ</t>
+          <t>SAUTE</t>
         </is>
       </c>
       <c r="D2">
-        <f>XLOOKUP(C2, tbl_Items[ItemCode], tbl_Items[ItemName], "")</f>
-        <v/>
-      </c>
-      <c r="E2" t="n">
-        <v>40</v>
-      </c>
-      <c r="F2">
-        <f>XLOOKUP(C2, tbl_Items[ItemCode], tbl_Items[PortionUOM], "")</f>
-        <v/>
+        <f>XLOOKUP(C2, tbl_Locations[LocationCode], tbl_Locations[LocationName], "")</f>
+        <v/>
+      </c>
+      <c r="E2">
+        <f>XLOOKUP(C2, tbl_Locations[LocationCode], tbl_Locations[PullPriority], 999)</f>
+        <v/>
+      </c>
+      <c r="F2" t="n">
+        <v>3</v>
       </c>
       <c r="G2">
-        <f>IFERROR(XLOOKUP(C2, tbl_Requisition[ItemCode], tbl_Requisition[TotalPortionsNeeded]), 0)</f>
+        <f>XLOOKUP(A2, tbl_Items[ItemCode], tbl_Items[PortionUOM], "")</f>
+        <v/>
+      </c>
+      <c r="H2">
+        <f>IFERROR(XLOOKUP(A2, tbl_Requisition[ItemCode], tbl_Requisition[TotalPortionsNeeded]), 0)</f>
+        <v/>
+      </c>
+      <c r="I2">
+        <f>SUMIFS(tbl_PullList[PortionsToPullHere], tbl_PullList[ItemCode], A2, tbl_PullList[PullPriority], "&lt;"&amp;E2)</f>
+        <v/>
+      </c>
+      <c r="J2">
+        <f>MIN(F2, MAX(0, H2-I2))</f>
+        <v/>
+      </c>
+      <c r="K2">
+        <f>MAX(0, H2-I2-J2)</f>
         <v/>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>FRZ</t>
+          <t>BUTTER</t>
         </is>
       </c>
       <c r="B3">
-        <f>XLOOKUP(A3, tbl_Locations[LocationCode], tbl_Locations[LocationName], "")</f>
+        <f>XLOOKUP(A3, tbl_Items[ItemCode], tbl_Items[ItemName], "")</f>
         <v/>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>PORK-CHOP-6OZ</t>
+          <t>WALKIN</t>
         </is>
       </c>
       <c r="D3">
-        <f>XLOOKUP(C3, tbl_Items[ItemCode], tbl_Items[ItemName], "")</f>
-        <v/>
-      </c>
-      <c r="E3" t="n">
-        <v>120</v>
-      </c>
-      <c r="F3">
-        <f>XLOOKUP(C3, tbl_Items[ItemCode], tbl_Items[PortionUOM], "")</f>
-        <v/>
+        <f>XLOOKUP(C3, tbl_Locations[LocationCode], tbl_Locations[LocationName], "")</f>
+        <v/>
+      </c>
+      <c r="E3">
+        <f>XLOOKUP(C3, tbl_Locations[LocationCode], tbl_Locations[PullPriority], 999)</f>
+        <v/>
+      </c>
+      <c r="F3" t="n">
+        <v>12</v>
       </c>
       <c r="G3">
-        <f>IFERROR(XLOOKUP(C3, tbl_Requisition[ItemCode], tbl_Requisition[TotalPortionsNeeded]), 0)</f>
+        <f>XLOOKUP(A3, tbl_Items[ItemCode], tbl_Items[PortionUOM], "")</f>
+        <v/>
+      </c>
+      <c r="H3">
+        <f>IFERROR(XLOOKUP(A3, tbl_Requisition[ItemCode], tbl_Requisition[TotalPortionsNeeded]), 0)</f>
+        <v/>
+      </c>
+      <c r="I3">
+        <f>SUMIFS(tbl_PullList[PortionsToPullHere], tbl_PullList[ItemCode], A3, tbl_PullList[PullPriority], "&lt;"&amp;E3)</f>
+        <v/>
+      </c>
+      <c r="J3">
+        <f>MIN(F3, MAX(0, H3-I3))</f>
+        <v/>
+      </c>
+      <c r="K3">
+        <f>MAX(0, H3-I3-J3)</f>
         <v/>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>PREP</t>
+          <t>CHIX-BRST-8OZ</t>
         </is>
       </c>
       <c r="B4">
-        <f>XLOOKUP(A4, tbl_Locations[LocationCode], tbl_Locations[LocationName], "")</f>
+        <f>XLOOKUP(A4, tbl_Items[ItemCode], tbl_Items[ItemName], "")</f>
         <v/>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>PORK-CHOP-6OZ</t>
+          <t>WALKIN</t>
         </is>
       </c>
       <c r="D4">
-        <f>XLOOKUP(C4, tbl_Items[ItemCode], tbl_Items[ItemName], "")</f>
-        <v/>
-      </c>
-      <c r="E4" t="n">
-        <v>8</v>
-      </c>
-      <c r="F4">
-        <f>XLOOKUP(C4, tbl_Items[ItemCode], tbl_Items[PortionUOM], "")</f>
-        <v/>
+        <f>XLOOKUP(C4, tbl_Locations[LocationCode], tbl_Locations[LocationName], "")</f>
+        <v/>
+      </c>
+      <c r="E4">
+        <f>XLOOKUP(C4, tbl_Locations[LocationCode], tbl_Locations[PullPriority], 999)</f>
+        <v/>
+      </c>
+      <c r="F4" t="n">
+        <v>32</v>
       </c>
       <c r="G4">
-        <f>IFERROR(XLOOKUP(C4, tbl_Requisition[ItemCode], tbl_Requisition[TotalPortionsNeeded]), 0)</f>
+        <f>XLOOKUP(A4, tbl_Items[ItemCode], tbl_Items[PortionUOM], "")</f>
+        <v/>
+      </c>
+      <c r="H4">
+        <f>IFERROR(XLOOKUP(A4, tbl_Requisition[ItemCode], tbl_Requisition[TotalPortionsNeeded]), 0)</f>
+        <v/>
+      </c>
+      <c r="I4">
+        <f>SUMIFS(tbl_PullList[PortionsToPullHere], tbl_PullList[ItemCode], A4, tbl_PullList[PullPriority], "&lt;"&amp;E4)</f>
+        <v/>
+      </c>
+      <c r="J4">
+        <f>MIN(F4, MAX(0, H4-I4))</f>
+        <v/>
+      </c>
+      <c r="K4">
+        <f>MAX(0, H4-I4-J4)</f>
         <v/>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>WALKIN</t>
+          <t>CHIX-BRST-8OZ</t>
         </is>
       </c>
       <c r="B5">
-        <f>XLOOKUP(A5, tbl_Locations[LocationCode], tbl_Locations[LocationName], "")</f>
+        <f>XLOOKUP(A5, tbl_Items[ItemCode], tbl_Items[ItemName], "")</f>
         <v/>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>CHIX-BRST-8OZ</t>
+          <t>FRZ</t>
         </is>
       </c>
       <c r="D5">
-        <f>XLOOKUP(C5, tbl_Items[ItemCode], tbl_Items[ItemName], "")</f>
-        <v/>
-      </c>
-      <c r="E5" t="n">
-        <v>32</v>
-      </c>
-      <c r="F5">
-        <f>XLOOKUP(C5, tbl_Items[ItemCode], tbl_Items[PortionUOM], "")</f>
-        <v/>
+        <f>XLOOKUP(C5, tbl_Locations[LocationCode], tbl_Locations[LocationName], "")</f>
+        <v/>
+      </c>
+      <c r="E5">
+        <f>XLOOKUP(C5, tbl_Locations[LocationCode], tbl_Locations[PullPriority], 999)</f>
+        <v/>
+      </c>
+      <c r="F5" t="n">
+        <v>80</v>
       </c>
       <c r="G5">
-        <f>IFERROR(XLOOKUP(C5, tbl_Requisition[ItemCode], tbl_Requisition[TotalPortionsNeeded]), 0)</f>
+        <f>XLOOKUP(A5, tbl_Items[ItemCode], tbl_Items[PortionUOM], "")</f>
+        <v/>
+      </c>
+      <c r="H5">
+        <f>IFERROR(XLOOKUP(A5, tbl_Requisition[ItemCode], tbl_Requisition[TotalPortionsNeeded]), 0)</f>
+        <v/>
+      </c>
+      <c r="I5">
+        <f>SUMIFS(tbl_PullList[PortionsToPullHere], tbl_PullList[ItemCode], A5, tbl_PullList[PullPriority], "&lt;"&amp;E5)</f>
+        <v/>
+      </c>
+      <c r="J5">
+        <f>MIN(F5, MAX(0, H5-I5))</f>
+        <v/>
+      </c>
+      <c r="K5">
+        <f>MAX(0, H5-I5-J5)</f>
         <v/>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>FRZ</t>
+          <t>CREAM-HVY</t>
         </is>
       </c>
       <c r="B6">
-        <f>XLOOKUP(A6, tbl_Locations[LocationCode], tbl_Locations[LocationName], "")</f>
+        <f>XLOOKUP(A6, tbl_Items[ItemCode], tbl_Items[ItemName], "")</f>
         <v/>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>CHIX-BRST-8OZ</t>
+          <t>WALKIN</t>
         </is>
       </c>
       <c r="D6">
-        <f>XLOOKUP(C6, tbl_Items[ItemCode], tbl_Items[ItemName], "")</f>
-        <v/>
-      </c>
-      <c r="E6" t="n">
-        <v>80</v>
-      </c>
-      <c r="F6">
-        <f>XLOOKUP(C6, tbl_Items[ItemCode], tbl_Items[PortionUOM], "")</f>
-        <v/>
+        <f>XLOOKUP(C6, tbl_Locations[LocationCode], tbl_Locations[LocationName], "")</f>
+        <v/>
+      </c>
+      <c r="E6">
+        <f>XLOOKUP(C6, tbl_Locations[LocationCode], tbl_Locations[PullPriority], 999)</f>
+        <v/>
+      </c>
+      <c r="F6" t="n">
+        <v>6</v>
       </c>
       <c r="G6">
-        <f>IFERROR(XLOOKUP(C6, tbl_Requisition[ItemCode], tbl_Requisition[TotalPortionsNeeded]), 0)</f>
+        <f>XLOOKUP(A6, tbl_Items[ItemCode], tbl_Items[PortionUOM], "")</f>
+        <v/>
+      </c>
+      <c r="H6">
+        <f>IFERROR(XLOOKUP(A6, tbl_Requisition[ItemCode], tbl_Requisition[TotalPortionsNeeded]), 0)</f>
+        <v/>
+      </c>
+      <c r="I6">
+        <f>SUMIFS(tbl_PullList[PortionsToPullHere], tbl_PullList[ItemCode], A6, tbl_PullList[PullPriority], "&lt;"&amp;E6)</f>
+        <v/>
+      </c>
+      <c r="J6">
+        <f>MIN(F6, MAX(0, H6-I6))</f>
+        <v/>
+      </c>
+      <c r="K6">
+        <f>MAX(0, H6-I6-J6)</f>
         <v/>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
+          <t>GARLIC</t>
+        </is>
+      </c>
+      <c r="B7">
+        <f>XLOOKUP(A7, tbl_Items[ItemCode], tbl_Items[ItemName], "")</f>
+        <v/>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
           <t>WALKIN</t>
         </is>
       </c>
-      <c r="B7">
-        <f>XLOOKUP(A7, tbl_Locations[LocationCode], tbl_Locations[LocationName], "")</f>
-        <v/>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>ONION-YEL</t>
-        </is>
-      </c>
       <c r="D7">
-        <f>XLOOKUP(C7, tbl_Items[ItemCode], tbl_Items[ItemName], "")</f>
-        <v/>
-      </c>
-      <c r="E7" t="n">
-        <v>18</v>
-      </c>
-      <c r="F7">
-        <f>XLOOKUP(C7, tbl_Items[ItemCode], tbl_Items[PortionUOM], "")</f>
-        <v/>
+        <f>XLOOKUP(C7, tbl_Locations[LocationCode], tbl_Locations[LocationName], "")</f>
+        <v/>
+      </c>
+      <c r="E7">
+        <f>XLOOKUP(C7, tbl_Locations[LocationCode], tbl_Locations[PullPriority], 999)</f>
+        <v/>
+      </c>
+      <c r="F7" t="n">
+        <v>15</v>
       </c>
       <c r="G7">
-        <f>IFERROR(XLOOKUP(C7, tbl_Requisition[ItemCode], tbl_Requisition[TotalPortionsNeeded]), 0)</f>
+        <f>XLOOKUP(A7, tbl_Items[ItemCode], tbl_Items[PortionUOM], "")</f>
+        <v/>
+      </c>
+      <c r="H7">
+        <f>IFERROR(XLOOKUP(A7, tbl_Requisition[ItemCode], tbl_Requisition[TotalPortionsNeeded]), 0)</f>
+        <v/>
+      </c>
+      <c r="I7">
+        <f>SUMIFS(tbl_PullList[PortionsToPullHere], tbl_PullList[ItemCode], A7, tbl_PullList[PullPriority], "&lt;"&amp;E7)</f>
+        <v/>
+      </c>
+      <c r="J7">
+        <f>MIN(F7, MAX(0, H7-I7))</f>
+        <v/>
+      </c>
+      <c r="K7">
+        <f>MAX(0, H7-I7-J7)</f>
         <v/>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>PREP</t>
+          <t>OIL-OLIVE</t>
         </is>
       </c>
       <c r="B8">
-        <f>XLOOKUP(A8, tbl_Locations[LocationCode], tbl_Locations[LocationName], "")</f>
+        <f>XLOOKUP(A8, tbl_Items[ItemCode], tbl_Items[ItemName], "")</f>
         <v/>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>ONION-YEL</t>
+          <t>DRY</t>
         </is>
       </c>
       <c r="D8">
-        <f>XLOOKUP(C8, tbl_Items[ItemCode], tbl_Items[ItemName], "")</f>
-        <v/>
-      </c>
-      <c r="E8" t="n">
-        <v>4</v>
-      </c>
-      <c r="F8">
-        <f>XLOOKUP(C8, tbl_Items[ItemCode], tbl_Items[PortionUOM], "")</f>
-        <v/>
+        <f>XLOOKUP(C8, tbl_Locations[LocationCode], tbl_Locations[LocationName], "")</f>
+        <v/>
+      </c>
+      <c r="E8">
+        <f>XLOOKUP(C8, tbl_Locations[LocationCode], tbl_Locations[PullPriority], 999)</f>
+        <v/>
+      </c>
+      <c r="F8" t="n">
+        <v>96</v>
       </c>
       <c r="G8">
-        <f>IFERROR(XLOOKUP(C8, tbl_Requisition[ItemCode], tbl_Requisition[TotalPortionsNeeded]), 0)</f>
+        <f>XLOOKUP(A8, tbl_Items[ItemCode], tbl_Items[PortionUOM], "")</f>
+        <v/>
+      </c>
+      <c r="H8">
+        <f>IFERROR(XLOOKUP(A8, tbl_Requisition[ItemCode], tbl_Requisition[TotalPortionsNeeded]), 0)</f>
+        <v/>
+      </c>
+      <c r="I8">
+        <f>SUMIFS(tbl_PullList[PortionsToPullHere], tbl_PullList[ItemCode], A8, tbl_PullList[PullPriority], "&lt;"&amp;E8)</f>
+        <v/>
+      </c>
+      <c r="J8">
+        <f>MIN(F8, MAX(0, H8-I8))</f>
+        <v/>
+      </c>
+      <c r="K8">
+        <f>MAX(0, H8-I8-J8)</f>
         <v/>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>WALKIN</t>
+          <t>ONION-YEL</t>
         </is>
       </c>
       <c r="B9">
-        <f>XLOOKUP(A9, tbl_Locations[LocationCode], tbl_Locations[LocationName], "")</f>
+        <f>XLOOKUP(A9, tbl_Items[ItemCode], tbl_Items[ItemName], "")</f>
         <v/>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>CREAM-HVY</t>
+          <t>PREP</t>
         </is>
       </c>
       <c r="D9">
-        <f>XLOOKUP(C9, tbl_Items[ItemCode], tbl_Items[ItemName], "")</f>
-        <v/>
-      </c>
-      <c r="E9" t="n">
-        <v>6</v>
-      </c>
-      <c r="F9">
-        <f>XLOOKUP(C9, tbl_Items[ItemCode], tbl_Items[PortionUOM], "")</f>
-        <v/>
+        <f>XLOOKUP(C9, tbl_Locations[LocationCode], tbl_Locations[LocationName], "")</f>
+        <v/>
+      </c>
+      <c r="E9">
+        <f>XLOOKUP(C9, tbl_Locations[LocationCode], tbl_Locations[PullPriority], 999)</f>
+        <v/>
+      </c>
+      <c r="F9" t="n">
+        <v>4</v>
       </c>
       <c r="G9">
-        <f>IFERROR(XLOOKUP(C9, tbl_Requisition[ItemCode], tbl_Requisition[TotalPortionsNeeded]), 0)</f>
+        <f>XLOOKUP(A9, tbl_Items[ItemCode], tbl_Items[PortionUOM], "")</f>
+        <v/>
+      </c>
+      <c r="H9">
+        <f>IFERROR(XLOOKUP(A9, tbl_Requisition[ItemCode], tbl_Requisition[TotalPortionsNeeded]), 0)</f>
+        <v/>
+      </c>
+      <c r="I9">
+        <f>SUMIFS(tbl_PullList[PortionsToPullHere], tbl_PullList[ItemCode], A9, tbl_PullList[PullPriority], "&lt;"&amp;E9)</f>
+        <v/>
+      </c>
+      <c r="J9">
+        <f>MIN(F9, MAX(0, H9-I9))</f>
+        <v/>
+      </c>
+      <c r="K9">
+        <f>MAX(0, H9-I9-J9)</f>
         <v/>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>DRY</t>
+          <t>ONION-YEL</t>
         </is>
       </c>
       <c r="B10">
-        <f>XLOOKUP(A10, tbl_Locations[LocationCode], tbl_Locations[LocationName], "")</f>
+        <f>XLOOKUP(A10, tbl_Items[ItemCode], tbl_Items[ItemName], "")</f>
         <v/>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>SALT-KOSHER</t>
+          <t>WALKIN</t>
         </is>
       </c>
       <c r="D10">
-        <f>XLOOKUP(C10, tbl_Items[ItemCode], tbl_Items[ItemName], "")</f>
-        <v/>
-      </c>
-      <c r="E10" t="n">
-        <v>720</v>
-      </c>
-      <c r="F10">
-        <f>XLOOKUP(C10, tbl_Items[ItemCode], tbl_Items[PortionUOM], "")</f>
-        <v/>
+        <f>XLOOKUP(C10, tbl_Locations[LocationCode], tbl_Locations[LocationName], "")</f>
+        <v/>
+      </c>
+      <c r="E10">
+        <f>XLOOKUP(C10, tbl_Locations[LocationCode], tbl_Locations[PullPriority], 999)</f>
+        <v/>
+      </c>
+      <c r="F10" t="n">
+        <v>18</v>
       </c>
       <c r="G10">
-        <f>IFERROR(XLOOKUP(C10, tbl_Requisition[ItemCode], tbl_Requisition[TotalPortionsNeeded]), 0)</f>
+        <f>XLOOKUP(A10, tbl_Items[ItemCode], tbl_Items[PortionUOM], "")</f>
+        <v/>
+      </c>
+      <c r="H10">
+        <f>IFERROR(XLOOKUP(A10, tbl_Requisition[ItemCode], tbl_Requisition[TotalPortionsNeeded]), 0)</f>
+        <v/>
+      </c>
+      <c r="I10">
+        <f>SUMIFS(tbl_PullList[PortionsToPullHere], tbl_PullList[ItemCode], A10, tbl_PullList[PullPriority], "&lt;"&amp;E10)</f>
+        <v/>
+      </c>
+      <c r="J10">
+        <f>MIN(F10, MAX(0, H10-I10))</f>
+        <v/>
+      </c>
+      <c r="K10">
+        <f>MAX(0, H10-I10-J10)</f>
         <v/>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>DRY</t>
+          <t>PARSLEY</t>
         </is>
       </c>
       <c r="B11">
-        <f>XLOOKUP(A11, tbl_Locations[LocationCode], tbl_Locations[LocationName], "")</f>
+        <f>XLOOKUP(A11, tbl_Items[ItemCode], tbl_Items[ItemName], "")</f>
         <v/>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>OIL-OLIVE</t>
+          <t>WALKIN</t>
         </is>
       </c>
       <c r="D11">
-        <f>XLOOKUP(C11, tbl_Items[ItemCode], tbl_Items[ItemName], "")</f>
-        <v/>
-      </c>
-      <c r="E11" t="n">
-        <v>96</v>
-      </c>
-      <c r="F11">
-        <f>XLOOKUP(C11, tbl_Items[ItemCode], tbl_Items[PortionUOM], "")</f>
-        <v/>
+        <f>XLOOKUP(C11, tbl_Locations[LocationCode], tbl_Locations[LocationName], "")</f>
+        <v/>
+      </c>
+      <c r="E11">
+        <f>XLOOKUP(C11, tbl_Locations[LocationCode], tbl_Locations[PullPriority], 999)</f>
+        <v/>
+      </c>
+      <c r="F11" t="n">
+        <v>4</v>
       </c>
       <c r="G11">
-        <f>IFERROR(XLOOKUP(C11, tbl_Requisition[ItemCode], tbl_Requisition[TotalPortionsNeeded]), 0)</f>
+        <f>XLOOKUP(A11, tbl_Items[ItemCode], tbl_Items[PortionUOM], "")</f>
+        <v/>
+      </c>
+      <c r="H11">
+        <f>IFERROR(XLOOKUP(A11, tbl_Requisition[ItemCode], tbl_Requisition[TotalPortionsNeeded]), 0)</f>
+        <v/>
+      </c>
+      <c r="I11">
+        <f>SUMIFS(tbl_PullList[PortionsToPullHere], tbl_PullList[ItemCode], A11, tbl_PullList[PullPriority], "&lt;"&amp;E11)</f>
+        <v/>
+      </c>
+      <c r="J11">
+        <f>MIN(F11, MAX(0, H11-I11))</f>
+        <v/>
+      </c>
+      <c r="K11">
+        <f>MAX(0, H11-I11-J11)</f>
         <v/>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>DRY</t>
+          <t>PORK-CHOP-6OZ</t>
         </is>
       </c>
       <c r="B12">
-        <f>XLOOKUP(A12, tbl_Locations[LocationCode], tbl_Locations[LocationName], "")</f>
+        <f>XLOOKUP(A12, tbl_Items[ItemCode], tbl_Items[ItemName], "")</f>
         <v/>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>POT-RUSSET</t>
+          <t>PREP</t>
         </is>
       </c>
       <c r="D12">
-        <f>XLOOKUP(C12, tbl_Items[ItemCode], tbl_Items[ItemName], "")</f>
-        <v/>
-      </c>
-      <c r="E12" t="n">
-        <v>48</v>
-      </c>
-      <c r="F12">
-        <f>XLOOKUP(C12, tbl_Items[ItemCode], tbl_Items[PortionUOM], "")</f>
-        <v/>
+        <f>XLOOKUP(C12, tbl_Locations[LocationCode], tbl_Locations[LocationName], "")</f>
+        <v/>
+      </c>
+      <c r="E12">
+        <f>XLOOKUP(C12, tbl_Locations[LocationCode], tbl_Locations[PullPriority], 999)</f>
+        <v/>
+      </c>
+      <c r="F12" t="n">
+        <v>8</v>
       </c>
       <c r="G12">
-        <f>IFERROR(XLOOKUP(C12, tbl_Requisition[ItemCode], tbl_Requisition[TotalPortionsNeeded]), 0)</f>
+        <f>XLOOKUP(A12, tbl_Items[ItemCode], tbl_Items[PortionUOM], "")</f>
+        <v/>
+      </c>
+      <c r="H12">
+        <f>IFERROR(XLOOKUP(A12, tbl_Requisition[ItemCode], tbl_Requisition[TotalPortionsNeeded]), 0)</f>
+        <v/>
+      </c>
+      <c r="I12">
+        <f>SUMIFS(tbl_PullList[PortionsToPullHere], tbl_PullList[ItemCode], A12, tbl_PullList[PullPriority], "&lt;"&amp;E12)</f>
+        <v/>
+      </c>
+      <c r="J12">
+        <f>MIN(F12, MAX(0, H12-I12))</f>
+        <v/>
+      </c>
+      <c r="K12">
+        <f>MAX(0, H12-I12-J12)</f>
         <v/>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>PREP</t>
+          <t>PORK-CHOP-6OZ</t>
         </is>
       </c>
       <c r="B13">
-        <f>XLOOKUP(A13, tbl_Locations[LocationCode], tbl_Locations[LocationName], "")</f>
+        <f>XLOOKUP(A13, tbl_Items[ItemCode], tbl_Items[ItemName], "")</f>
         <v/>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>POT-RUSSET</t>
+          <t>WALKIN</t>
         </is>
       </c>
       <c r="D13">
-        <f>XLOOKUP(C13, tbl_Items[ItemCode], tbl_Items[ItemName], "")</f>
-        <v/>
-      </c>
-      <c r="E13" t="n">
-        <v>10</v>
-      </c>
-      <c r="F13">
-        <f>XLOOKUP(C13, tbl_Items[ItemCode], tbl_Items[PortionUOM], "")</f>
-        <v/>
+        <f>XLOOKUP(C13, tbl_Locations[LocationCode], tbl_Locations[LocationName], "")</f>
+        <v/>
+      </c>
+      <c r="E13">
+        <f>XLOOKUP(C13, tbl_Locations[LocationCode], tbl_Locations[PullPriority], 999)</f>
+        <v/>
+      </c>
+      <c r="F13" t="n">
+        <v>40</v>
       </c>
       <c r="G13">
-        <f>IFERROR(XLOOKUP(C13, tbl_Requisition[ItemCode], tbl_Requisition[TotalPortionsNeeded]), 0)</f>
+        <f>XLOOKUP(A13, tbl_Items[ItemCode], tbl_Items[PortionUOM], "")</f>
+        <v/>
+      </c>
+      <c r="H13">
+        <f>IFERROR(XLOOKUP(A13, tbl_Requisition[ItemCode], tbl_Requisition[TotalPortionsNeeded]), 0)</f>
+        <v/>
+      </c>
+      <c r="I13">
+        <f>SUMIFS(tbl_PullList[PortionsToPullHere], tbl_PullList[ItemCode], A13, tbl_PullList[PullPriority], "&lt;"&amp;E13)</f>
+        <v/>
+      </c>
+      <c r="J13">
+        <f>MIN(F13, MAX(0, H13-I13))</f>
+        <v/>
+      </c>
+      <c r="K13">
+        <f>MAX(0, H13-I13-J13)</f>
         <v/>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>WALKIN</t>
+          <t>PORK-CHOP-6OZ</t>
         </is>
       </c>
       <c r="B14">
-        <f>XLOOKUP(A14, tbl_Locations[LocationCode], tbl_Locations[LocationName], "")</f>
+        <f>XLOOKUP(A14, tbl_Items[ItemCode], tbl_Items[ItemName], "")</f>
         <v/>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>BUTTER</t>
+          <t>FRZ</t>
         </is>
       </c>
       <c r="D14">
-        <f>XLOOKUP(C14, tbl_Items[ItemCode], tbl_Items[ItemName], "")</f>
-        <v/>
-      </c>
-      <c r="E14" t="n">
-        <v>12</v>
-      </c>
-      <c r="F14">
-        <f>XLOOKUP(C14, tbl_Items[ItemCode], tbl_Items[PortionUOM], "")</f>
-        <v/>
+        <f>XLOOKUP(C14, tbl_Locations[LocationCode], tbl_Locations[LocationName], "")</f>
+        <v/>
+      </c>
+      <c r="E14">
+        <f>XLOOKUP(C14, tbl_Locations[LocationCode], tbl_Locations[PullPriority], 999)</f>
+        <v/>
+      </c>
+      <c r="F14" t="n">
+        <v>120</v>
       </c>
       <c r="G14">
-        <f>IFERROR(XLOOKUP(C14, tbl_Requisition[ItemCode], tbl_Requisition[TotalPortionsNeeded]), 0)</f>
+        <f>XLOOKUP(A14, tbl_Items[ItemCode], tbl_Items[PortionUOM], "")</f>
+        <v/>
+      </c>
+      <c r="H14">
+        <f>IFERROR(XLOOKUP(A14, tbl_Requisition[ItemCode], tbl_Requisition[TotalPortionsNeeded]), 0)</f>
+        <v/>
+      </c>
+      <c r="I14">
+        <f>SUMIFS(tbl_PullList[PortionsToPullHere], tbl_PullList[ItemCode], A14, tbl_PullList[PullPriority], "&lt;"&amp;E14)</f>
+        <v/>
+      </c>
+      <c r="J14">
+        <f>MIN(F14, MAX(0, H14-I14))</f>
+        <v/>
+      </c>
+      <c r="K14">
+        <f>MAX(0, H14-I14-J14)</f>
         <v/>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>SAUTE</t>
+          <t>POT-RUSSET</t>
         </is>
       </c>
       <c r="B15">
-        <f>XLOOKUP(A15, tbl_Locations[LocationCode], tbl_Locations[LocationName], "")</f>
+        <f>XLOOKUP(A15, tbl_Items[ItemCode], tbl_Items[ItemName], "")</f>
         <v/>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>BUTTER</t>
+          <t>PREP</t>
         </is>
       </c>
       <c r="D15">
-        <f>XLOOKUP(C15, tbl_Items[ItemCode], tbl_Items[ItemName], "")</f>
-        <v/>
-      </c>
-      <c r="E15" t="n">
-        <v>3</v>
-      </c>
-      <c r="F15">
-        <f>XLOOKUP(C15, tbl_Items[ItemCode], tbl_Items[PortionUOM], "")</f>
-        <v/>
+        <f>XLOOKUP(C15, tbl_Locations[LocationCode], tbl_Locations[LocationName], "")</f>
+        <v/>
+      </c>
+      <c r="E15">
+        <f>XLOOKUP(C15, tbl_Locations[LocationCode], tbl_Locations[PullPriority], 999)</f>
+        <v/>
+      </c>
+      <c r="F15" t="n">
+        <v>10</v>
       </c>
       <c r="G15">
-        <f>IFERROR(XLOOKUP(C15, tbl_Requisition[ItemCode], tbl_Requisition[TotalPortionsNeeded]), 0)</f>
+        <f>XLOOKUP(A15, tbl_Items[ItemCode], tbl_Items[PortionUOM], "")</f>
+        <v/>
+      </c>
+      <c r="H15">
+        <f>IFERROR(XLOOKUP(A15, tbl_Requisition[ItemCode], tbl_Requisition[TotalPortionsNeeded]), 0)</f>
+        <v/>
+      </c>
+      <c r="I15">
+        <f>SUMIFS(tbl_PullList[PortionsToPullHere], tbl_PullList[ItemCode], A15, tbl_PullList[PullPriority], "&lt;"&amp;E15)</f>
+        <v/>
+      </c>
+      <c r="J15">
+        <f>MIN(F15, MAX(0, H15-I15))</f>
+        <v/>
+      </c>
+      <c r="K15">
+        <f>MAX(0, H15-I15-J15)</f>
         <v/>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>WALKIN</t>
+          <t>POT-RUSSET</t>
         </is>
       </c>
       <c r="B16">
-        <f>XLOOKUP(A16, tbl_Locations[LocationCode], tbl_Locations[LocationName], "")</f>
+        <f>XLOOKUP(A16, tbl_Items[ItemCode], tbl_Items[ItemName], "")</f>
         <v/>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>GARLIC</t>
+          <t>DRY</t>
         </is>
       </c>
       <c r="D16">
-        <f>XLOOKUP(C16, tbl_Items[ItemCode], tbl_Items[ItemName], "")</f>
-        <v/>
-      </c>
-      <c r="E16" t="n">
-        <v>15</v>
-      </c>
-      <c r="F16">
-        <f>XLOOKUP(C16, tbl_Items[ItemCode], tbl_Items[PortionUOM], "")</f>
-        <v/>
+        <f>XLOOKUP(C16, tbl_Locations[LocationCode], tbl_Locations[LocationName], "")</f>
+        <v/>
+      </c>
+      <c r="E16">
+        <f>XLOOKUP(C16, tbl_Locations[LocationCode], tbl_Locations[PullPriority], 999)</f>
+        <v/>
+      </c>
+      <c r="F16" t="n">
+        <v>48</v>
       </c>
       <c r="G16">
-        <f>IFERROR(XLOOKUP(C16, tbl_Requisition[ItemCode], tbl_Requisition[TotalPortionsNeeded]), 0)</f>
+        <f>XLOOKUP(A16, tbl_Items[ItemCode], tbl_Items[PortionUOM], "")</f>
+        <v/>
+      </c>
+      <c r="H16">
+        <f>IFERROR(XLOOKUP(A16, tbl_Requisition[ItemCode], tbl_Requisition[TotalPortionsNeeded]), 0)</f>
+        <v/>
+      </c>
+      <c r="I16">
+        <f>SUMIFS(tbl_PullList[PortionsToPullHere], tbl_PullList[ItemCode], A16, tbl_PullList[PullPriority], "&lt;"&amp;E16)</f>
+        <v/>
+      </c>
+      <c r="J16">
+        <f>MIN(F16, MAX(0, H16-I16))</f>
+        <v/>
+      </c>
+      <c r="K16">
+        <f>MAX(0, H16-I16-J16)</f>
         <v/>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>WALKIN</t>
+          <t>SALT-KOSHER</t>
         </is>
       </c>
       <c r="B17">
-        <f>XLOOKUP(A17, tbl_Locations[LocationCode], tbl_Locations[LocationName], "")</f>
+        <f>XLOOKUP(A17, tbl_Items[ItemCode], tbl_Items[ItemName], "")</f>
         <v/>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>PARSLEY</t>
+          <t>DRY</t>
         </is>
       </c>
       <c r="D17">
-        <f>XLOOKUP(C17, tbl_Items[ItemCode], tbl_Items[ItemName], "")</f>
-        <v/>
-      </c>
-      <c r="E17" t="n">
-        <v>4</v>
-      </c>
-      <c r="F17">
-        <f>XLOOKUP(C17, tbl_Items[ItemCode], tbl_Items[PortionUOM], "")</f>
-        <v/>
+        <f>XLOOKUP(C17, tbl_Locations[LocationCode], tbl_Locations[LocationName], "")</f>
+        <v/>
+      </c>
+      <c r="E17">
+        <f>XLOOKUP(C17, tbl_Locations[LocationCode], tbl_Locations[PullPriority], 999)</f>
+        <v/>
+      </c>
+      <c r="F17" t="n">
+        <v>720</v>
       </c>
       <c r="G17">
-        <f>IFERROR(XLOOKUP(C17, tbl_Requisition[ItemCode], tbl_Requisition[TotalPortionsNeeded]), 0)</f>
+        <f>XLOOKUP(A17, tbl_Items[ItemCode], tbl_Items[PortionUOM], "")</f>
+        <v/>
+      </c>
+      <c r="H17">
+        <f>IFERROR(XLOOKUP(A17, tbl_Requisition[ItemCode], tbl_Requisition[TotalPortionsNeeded]), 0)</f>
+        <v/>
+      </c>
+      <c r="I17">
+        <f>SUMIFS(tbl_PullList[PortionsToPullHere], tbl_PullList[ItemCode], A17, tbl_PullList[PullPriority], "&lt;"&amp;E17)</f>
+        <v/>
+      </c>
+      <c r="J17">
+        <f>MIN(F17, MAX(0, H17-I17))</f>
+        <v/>
+      </c>
+      <c r="K17">
+        <f>MAX(0, H17-I17-J17)</f>
         <v/>
       </c>
     </row>

</xml_diff>